<commit_message>
fix(phones,exports): To'liq telefonlarni tozalash, 2-raqamni ajratish, debitorka shartnomalari va rollar eksportini yangilash
</commit_message>
<xml_diff>
--- a/data/Talabalar_Yangilangan_Royxat.xlsx
+++ b/data/Talabalar_Yangilangan_Royxat.xlsx
@@ -791,7 +791,11 @@
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>303</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="inlineStr">
         <is>
@@ -875,7 +879,11 @@
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr"/>
-      <c r="E3" s="11" t="inlineStr"/>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
       <c r="F3" s="11" t="inlineStr"/>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -959,7 +967,11 @@
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>274</t>
+        </is>
+      </c>
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -1043,7 +1055,11 @@
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr"/>
-      <c r="E5" s="11" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>286</t>
+        </is>
+      </c>
       <c r="F5" s="11" t="inlineStr"/>
       <c r="G5" s="11" t="inlineStr">
         <is>
@@ -1133,7 +1149,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>140</t>
         </is>
       </c>
       <c r="F6" s="12" t="n">
@@ -1200,8 +1216,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T6" s="5" t="n">
-        <v>2026</v>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>+998 88 848-08-27 / +998 97 855-05-81 (Onasi)</t>
+        </is>
       </c>
       <c r="U6" s="7" t="inlineStr">
         <is>
@@ -1239,7 +1257,11 @@
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr"/>
-      <c r="E7" s="11" t="inlineStr"/>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
       <c r="F7" s="11" t="inlineStr"/>
       <c r="G7" s="11" t="inlineStr">
         <is>
@@ -1329,7 +1351,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>204</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -1400,7 +1422,7 @@
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>+998 18 980-49-50 / +998 08 830-86-50 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U8" s="7" t="inlineStr">
@@ -1439,7 +1461,11 @@
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr"/>
-      <c r="E9" s="11" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="F9" s="11" t="inlineStr"/>
       <c r="G9" s="11" t="inlineStr">
         <is>
@@ -1531,7 +1557,11 @@
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>312</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
@@ -1617,7 +1647,7 @@
       <c r="D11" s="10" t="inlineStr"/>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>272</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -1692,7 +1722,7 @@
       </c>
       <c r="T11" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 871-57-37</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -1727,7 +1757,11 @@
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -1817,7 +1851,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>79</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -1892,7 +1926,7 @@
       </c>
       <c r="T13" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 03 318-70-80 / +998 01 190-68-60 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
@@ -1933,7 +1967,7 @@
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>286</t>
+          <t>224</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -2008,7 +2042,7 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 905-47-05 / +998 99 419-23-74 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U14" s="7" t="inlineStr">
@@ -2053,7 +2087,7 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>258</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
@@ -2128,7 +2162,7 @@
       </c>
       <c r="T15" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 463-62-67</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
@@ -2163,7 +2197,11 @@
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
       <c r="F16" s="5" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
@@ -2247,7 +2285,11 @@
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr"/>
-      <c r="E17" s="11" t="inlineStr"/>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
       <c r="F17" s="11" t="inlineStr"/>
       <c r="G17" s="11" t="inlineStr">
         <is>
@@ -2335,7 +2377,11 @@
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="F18" s="5" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr">
         <is>
@@ -2419,7 +2465,11 @@
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr"/>
-      <c r="E19" s="11" t="inlineStr"/>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="F19" s="11" t="inlineStr"/>
       <c r="G19" s="11" t="inlineStr">
         <is>
@@ -2507,7 +2557,11 @@
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
       <c r="F20" s="5" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
@@ -2597,7 +2651,7 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>109</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
@@ -2672,7 +2726,7 @@
       </c>
       <c r="T21" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 90 243-37-74 / +998 88 588-81-87 (Onasi)</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
@@ -2707,7 +2761,11 @@
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
@@ -2797,7 +2855,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>123</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
@@ -2872,7 +2930,7 @@
       </c>
       <c r="T23" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 75 910-91-80 / +998 88 566-08-02 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
@@ -2907,7 +2965,11 @@
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
@@ -2997,7 +3059,7 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>174</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
@@ -3072,7 +3134,7 @@
       </c>
       <c r="T25" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 99 221-68-64 / +998 93 666-02-15 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
@@ -3107,7 +3169,11 @@
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="5" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
       <c r="F26" s="5" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
@@ -3191,7 +3257,11 @@
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr"/>
-      <c r="E27" s="11" t="inlineStr"/>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
       <c r="F27" s="11" t="inlineStr"/>
       <c r="G27" s="11" t="inlineStr">
         <is>
@@ -3277,7 +3347,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -3340,7 +3410,7 @@
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 00 343-13-10</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
@@ -3373,7 +3443,7 @@
       <c r="D29" s="10" t="inlineStr"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>267</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
@@ -3442,11 +3512,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T29" s="11" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
+      <c r="T29" s="11" t="inlineStr"/>
       <c r="U29" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -3483,7 +3549,11 @@
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
@@ -3567,7 +3637,11 @@
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr"/>
-      <c r="E31" s="11" t="inlineStr"/>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>381</t>
+        </is>
+      </c>
       <c r="F31" s="11" t="inlineStr"/>
       <c r="G31" s="11" t="inlineStr">
         <is>
@@ -3651,7 +3725,11 @@
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
@@ -3731,7 +3809,11 @@
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr"/>
-      <c r="E33" s="11" t="inlineStr"/>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
       <c r="F33" s="11" t="inlineStr"/>
       <c r="G33" s="11" t="inlineStr">
         <is>
@@ -3815,7 +3897,11 @@
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
       <c r="F34" s="5" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
@@ -3905,7 +3991,7 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>182</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
@@ -3980,7 +4066,7 @@
       </c>
       <c r="T35" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 95 367-26-02 / +998 90 616-15-60 (Buvasi)</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
@@ -4017,7 +4103,7 @@
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>278</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -4090,11 +4176,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T36" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
+      <c r="T36" s="5" t="inlineStr"/>
       <c r="U36" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -4127,7 +4209,11 @@
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr"/>
-      <c r="E37" s="11" t="inlineStr"/>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>275</t>
+        </is>
+      </c>
       <c r="F37" s="11" t="inlineStr"/>
       <c r="G37" s="11" t="inlineStr">
         <is>
@@ -4217,7 +4303,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>166</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -4292,7 +4378,7 @@
       </c>
       <c r="T38" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 91 219-06-17 / +998 91 217-34-81 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U38" s="7" t="inlineStr">
@@ -4327,7 +4413,11 @@
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr"/>
-      <c r="E39" s="11" t="inlineStr"/>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
       <c r="F39" s="11" t="inlineStr"/>
       <c r="G39" s="11" t="inlineStr">
         <is>
@@ -4411,7 +4501,11 @@
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
       <c r="F40" s="5" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr">
         <is>
@@ -4495,7 +4589,11 @@
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr"/>
-      <c r="E41" s="11" t="inlineStr"/>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
       <c r="F41" s="11" t="inlineStr"/>
       <c r="G41" s="11" t="inlineStr">
         <is>
@@ -4579,7 +4677,11 @@
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>292</t>
+        </is>
+      </c>
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
@@ -4663,7 +4765,11 @@
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr"/>
-      <c r="E43" s="11" t="inlineStr"/>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
       <c r="F43" s="11" t="inlineStr"/>
       <c r="G43" s="11" t="inlineStr">
         <is>
@@ -4753,7 +4859,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>258</t>
+          <t>294</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -4816,7 +4922,7 @@
       </c>
       <c r="T44" s="5" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>+998 91 957-18-58</t>
         </is>
       </c>
       <c r="U44" s="15" t="inlineStr">
@@ -4851,7 +4957,11 @@
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr"/>
-      <c r="E45" s="11" t="inlineStr"/>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
       <c r="F45" s="11" t="inlineStr"/>
       <c r="G45" s="11" t="inlineStr">
         <is>
@@ -4945,7 +5055,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>65</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -5020,7 +5130,7 @@
       </c>
       <c r="T46" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 70 120-22-08 / +998 70 125-22-08 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U46" s="7" t="inlineStr">
@@ -5061,7 +5171,7 @@
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>383</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
@@ -5136,7 +5246,7 @@
       </c>
       <c r="T47" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 312-50-80 / +998 76 078-28-70 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
@@ -5177,7 +5287,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>318</t>
+          <t>202</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr"/>
@@ -5244,7 +5354,7 @@
       </c>
       <c r="T48" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 97 799-76-71 / +998 88 403-76-71 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U48" s="15" t="inlineStr">
@@ -5275,7 +5385,11 @@
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr"/>
-      <c r="E49" s="11" t="inlineStr"/>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
       <c r="F49" s="11" t="inlineStr"/>
       <c r="G49" s="11" t="inlineStr">
         <is>
@@ -5365,7 +5479,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -5440,7 +5554,7 @@
       </c>
       <c r="T50" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 77 602-17-08 / +998 70 219-11-08 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U50" s="7" t="inlineStr">
@@ -5475,7 +5589,11 @@
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr"/>
-      <c r="E51" s="11" t="inlineStr"/>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
       <c r="F51" s="11" t="inlineStr"/>
       <c r="G51" s="11" t="inlineStr">
         <is>
@@ -5559,7 +5677,11 @@
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr"/>
-      <c r="E52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>262</t>
+        </is>
+      </c>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr">
         <is>
@@ -5643,7 +5765,11 @@
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr"/>
-      <c r="E53" s="11" t="inlineStr"/>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
       <c r="F53" s="11" t="inlineStr"/>
       <c r="G53" s="11" t="inlineStr">
         <is>
@@ -5727,7 +5853,11 @@
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr"/>
-      <c r="E54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="inlineStr">
         <is>
@@ -5811,7 +5941,11 @@
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr"/>
-      <c r="E55" s="11" t="inlineStr"/>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="F55" s="11" t="inlineStr"/>
       <c r="G55" s="11" t="inlineStr">
         <is>
@@ -5895,7 +6029,11 @@
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr"/>
-      <c r="E56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="5" t="inlineStr">
         <is>
@@ -5979,7 +6117,11 @@
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr"/>
-      <c r="E57" s="11" t="inlineStr"/>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
       <c r="F57" s="11" t="inlineStr"/>
       <c r="G57" s="11" t="inlineStr">
         <is>
@@ -6063,7 +6205,11 @@
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr"/>
-      <c r="E58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="5" t="inlineStr">
         <is>
@@ -6147,7 +6293,11 @@
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr"/>
-      <c r="E59" s="11" t="inlineStr"/>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>293</t>
+        </is>
+      </c>
       <c r="F59" s="11" t="inlineStr"/>
       <c r="G59" s="11" t="inlineStr">
         <is>
@@ -6233,7 +6383,7 @@
       <c r="D60" s="4" t="inlineStr"/>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>139</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -6308,7 +6458,7 @@
       </c>
       <c r="T60" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 77 432-17-07 / +998 95 616-35-09 (Onasi)</t>
         </is>
       </c>
       <c r="U60" s="7" t="inlineStr">
@@ -6347,7 +6497,11 @@
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr"/>
-      <c r="E61" s="11" t="inlineStr"/>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>390</t>
+        </is>
+      </c>
       <c r="F61" s="11" t="inlineStr"/>
       <c r="G61" s="11" t="inlineStr">
         <is>
@@ -6437,7 +6591,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>314</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -6508,7 +6662,7 @@
       </c>
       <c r="T62" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>+998 70 629-89-00 / +998 97 319-62-60 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U62" s="7" t="inlineStr">
@@ -6543,7 +6697,11 @@
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr"/>
-      <c r="E63" s="11" t="inlineStr"/>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>277</t>
+        </is>
+      </c>
       <c r="F63" s="11" t="inlineStr"/>
       <c r="G63" s="11" t="inlineStr">
         <is>
@@ -6627,7 +6785,11 @@
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr"/>
-      <c r="E64" s="5" t="inlineStr"/>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
       <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr">
         <is>
@@ -6711,7 +6873,11 @@
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr"/>
-      <c r="E65" s="11" t="inlineStr"/>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="F65" s="11" t="inlineStr"/>
       <c r="G65" s="11" t="inlineStr">
         <is>
@@ -6795,7 +6961,11 @@
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr"/>
-      <c r="E66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr">
         <is>
@@ -6875,7 +7045,11 @@
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr"/>
-      <c r="E67" s="11" t="inlineStr"/>
+      <c r="E67" s="11" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
       <c r="F67" s="11" t="inlineStr"/>
       <c r="G67" s="11" t="inlineStr">
         <is>
@@ -6959,7 +7133,11 @@
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr"/>
-      <c r="E68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
       <c r="F68" s="5" t="inlineStr"/>
       <c r="G68" s="5" t="inlineStr">
         <is>
@@ -7039,7 +7217,11 @@
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr"/>
-      <c r="E69" s="11" t="inlineStr"/>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
       <c r="F69" s="11" t="inlineStr"/>
       <c r="G69" s="11" t="inlineStr">
         <is>
@@ -7123,7 +7305,11 @@
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr"/>
-      <c r="E70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="F70" s="5" t="inlineStr"/>
       <c r="G70" s="5" t="inlineStr">
         <is>
@@ -7211,7 +7397,11 @@
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr"/>
-      <c r="E71" s="11" t="inlineStr"/>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="F71" s="11" t="inlineStr"/>
       <c r="G71" s="11" t="inlineStr">
         <is>
@@ -7295,7 +7485,11 @@
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr"/>
-      <c r="E72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="F72" s="5" t="inlineStr"/>
       <c r="G72" s="5" t="inlineStr">
         <is>
@@ -7379,7 +7573,11 @@
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr"/>
-      <c r="E73" s="11" t="inlineStr"/>
+      <c r="E73" s="11" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
       <c r="F73" s="11" t="inlineStr"/>
       <c r="G73" s="11" t="inlineStr">
         <is>
@@ -7551,7 +7749,11 @@
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr"/>
-      <c r="E75" s="11" t="inlineStr"/>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>163</t>
+        </is>
+      </c>
       <c r="F75" s="11" t="inlineStr"/>
       <c r="G75" s="11" t="inlineStr">
         <is>
@@ -7639,7 +7841,11 @@
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr"/>
-      <c r="E76" s="5" t="inlineStr"/>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
       <c r="F76" s="5" t="inlineStr"/>
       <c r="G76" s="5" t="inlineStr">
         <is>
@@ -7723,7 +7929,11 @@
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr"/>
-      <c r="E77" s="11" t="inlineStr"/>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
       <c r="F77" s="11" t="inlineStr"/>
       <c r="G77" s="11" t="inlineStr">
         <is>
@@ -7807,7 +8017,11 @@
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr"/>
-      <c r="E78" s="5" t="inlineStr"/>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
       <c r="F78" s="5" t="inlineStr"/>
       <c r="G78" s="5" t="inlineStr">
         <is>
@@ -7895,7 +8109,11 @@
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr"/>
-      <c r="E79" s="11" t="inlineStr"/>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="F79" s="11" t="inlineStr"/>
       <c r="G79" s="11" t="inlineStr">
         <is>
@@ -7981,7 +8199,7 @@
       <c r="D80" s="4" t="inlineStr"/>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>282</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
@@ -8052,7 +8270,7 @@
       </c>
       <c r="T80" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 88 309-02-28 / +998 88 005-78-08 (Onasi)</t>
         </is>
       </c>
       <c r="U80" s="7" t="inlineStr">
@@ -8087,7 +8305,11 @@
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr"/>
-      <c r="E81" s="11" t="inlineStr"/>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
       <c r="F81" s="11" t="inlineStr"/>
       <c r="G81" s="11" t="inlineStr">
         <is>
@@ -8177,7 +8399,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>176</t>
         </is>
       </c>
       <c r="F82" s="12" t="n">
@@ -8244,8 +8466,10 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="T82" s="5" t="n">
-        <v>2014</v>
+      <c r="T82" s="5" t="inlineStr">
+        <is>
+          <t>+998 88 788-60-42 / +998 88 308-60-42 (Otasi / Onasi)</t>
+        </is>
       </c>
       <c r="U82" s="7" t="inlineStr">
         <is>
@@ -8283,7 +8507,11 @@
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr"/>
-      <c r="E83" s="11" t="inlineStr"/>
+      <c r="E83" s="11" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
       <c r="F83" s="11" t="inlineStr"/>
       <c r="G83" s="11" t="inlineStr">
         <is>
@@ -8367,7 +8595,11 @@
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr"/>
-      <c r="E84" s="5" t="inlineStr"/>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
+      </c>
       <c r="F84" s="5" t="inlineStr"/>
       <c r="G84" s="5" t="inlineStr">
         <is>
@@ -8451,7 +8683,11 @@
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr"/>
-      <c r="E85" s="11" t="inlineStr"/>
+      <c r="E85" s="11" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="F85" s="11" t="inlineStr"/>
       <c r="G85" s="11" t="inlineStr">
         <is>
@@ -8535,7 +8771,11 @@
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr"/>
-      <c r="E86" s="5" t="inlineStr"/>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>258</t>
+        </is>
+      </c>
       <c r="F86" s="5" t="inlineStr"/>
       <c r="G86" s="5" t="inlineStr">
         <is>
@@ -8787,7 +9027,11 @@
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr"/>
-      <c r="E89" s="11" t="inlineStr"/>
+      <c r="E89" s="11" t="inlineStr">
+        <is>
+          <t>304</t>
+        </is>
+      </c>
       <c r="F89" s="11" t="inlineStr"/>
       <c r="G89" s="11" t="inlineStr">
         <is>
@@ -8871,7 +9115,11 @@
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr"/>
-      <c r="E90" s="5" t="inlineStr"/>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
       <c r="F90" s="5" t="inlineStr"/>
       <c r="G90" s="5" t="inlineStr">
         <is>
@@ -8955,7 +9203,11 @@
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr"/>
-      <c r="E91" s="11" t="inlineStr"/>
+      <c r="E91" s="11" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
       <c r="F91" s="11" t="inlineStr"/>
       <c r="G91" s="11" t="inlineStr">
         <is>
@@ -9043,7 +9295,11 @@
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr"/>
-      <c r="E92" s="5" t="inlineStr"/>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
       <c r="F92" s="5" t="inlineStr"/>
       <c r="G92" s="5" t="inlineStr">
         <is>
@@ -9129,7 +9385,7 @@
       <c r="D93" s="10" t="inlineStr"/>
       <c r="E93" s="11" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F93" s="11" t="inlineStr">
@@ -9200,7 +9456,7 @@
       </c>
       <c r="T93" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 768-70-08</t>
         </is>
       </c>
       <c r="U93" s="7" t="inlineStr">
@@ -9239,7 +9495,11 @@
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr"/>
-      <c r="E94" s="5" t="inlineStr"/>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
       <c r="F94" s="5" t="inlineStr"/>
       <c r="G94" s="5" t="inlineStr">
         <is>
@@ -9323,7 +9583,11 @@
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr"/>
-      <c r="E95" s="11" t="inlineStr"/>
+      <c r="E95" s="11" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
       <c r="F95" s="11" t="inlineStr"/>
       <c r="G95" s="11" t="inlineStr">
         <is>
@@ -9413,7 +9677,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>230</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
@@ -9484,7 +9748,7 @@
       </c>
       <c r="T96" s="5" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>+998 88 097-94-77</t>
         </is>
       </c>
       <c r="U96" s="7" t="inlineStr">
@@ -9609,7 +9873,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -9676,7 +9940,7 @@
       </c>
       <c r="T98" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 77 042-82-25</t>
         </is>
       </c>
       <c r="U98" s="15" t="inlineStr">
@@ -9711,7 +9975,11 @@
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr"/>
-      <c r="E99" s="11" t="inlineStr"/>
+      <c r="E99" s="11" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
       <c r="F99" s="11" t="inlineStr"/>
       <c r="G99" s="11" t="inlineStr">
         <is>
@@ -9791,7 +10059,11 @@
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr"/>
-      <c r="E100" s="5" t="inlineStr"/>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="F100" s="5" t="inlineStr"/>
       <c r="G100" s="5" t="inlineStr">
         <is>
@@ -9875,7 +10147,11 @@
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr"/>
-      <c r="E101" s="11" t="inlineStr"/>
+      <c r="E101" s="11" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
       <c r="F101" s="11" t="inlineStr"/>
       <c r="G101" s="11" t="inlineStr">
         <is>
@@ -9955,7 +10231,11 @@
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr"/>
-      <c r="E102" s="5" t="inlineStr"/>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="F102" s="5" t="inlineStr"/>
       <c r="G102" s="5" t="inlineStr">
         <is>
@@ -10045,7 +10325,7 @@
       </c>
       <c r="E103" s="11" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>251</t>
         </is>
       </c>
       <c r="F103" s="11" t="inlineStr">
@@ -10120,7 +10400,7 @@
       </c>
       <c r="T103" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 619-02-15</t>
         </is>
       </c>
       <c r="U103" s="7" t="inlineStr">
@@ -10157,7 +10437,7 @@
       <c r="D104" s="4" t="inlineStr"/>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -10224,7 +10504,7 @@
       </c>
       <c r="T104" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 709-08-76</t>
         </is>
       </c>
       <c r="U104" s="17" t="inlineStr">
@@ -10259,7 +10539,11 @@
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr"/>
-      <c r="E105" s="11" t="inlineStr"/>
+      <c r="E105" s="11" t="inlineStr">
+        <is>
+          <t>295</t>
+        </is>
+      </c>
       <c r="F105" s="11" t="inlineStr"/>
       <c r="G105" s="11" t="inlineStr">
         <is>
@@ -10349,7 +10633,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>187</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -10424,7 +10708,7 @@
       </c>
       <c r="T106" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 76 310-47-70 / +998 73 210-47-70 (Turmush o'rtog'i)</t>
         </is>
       </c>
       <c r="U106" s="7" t="inlineStr">
@@ -10459,7 +10743,11 @@
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr"/>
-      <c r="E107" s="11" t="inlineStr"/>
+      <c r="E107" s="11" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
       <c r="F107" s="11" t="inlineStr"/>
       <c r="G107" s="11" t="inlineStr">
         <is>
@@ -10545,7 +10833,7 @@
       <c r="D108" s="4" t="inlineStr"/>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>267</t>
+          <t>392</t>
         </is>
       </c>
       <c r="F108" s="12" t="n">
@@ -10612,8 +10900,10 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="T108" s="5" t="n">
-        <v>2017</v>
+      <c r="T108" s="5" t="inlineStr">
+        <is>
+          <t>+998 99 186-30-23 / +998 99 186-30-23 (O'zi)</t>
+        </is>
       </c>
       <c r="U108" s="7" t="inlineStr">
         <is>
@@ -10647,7 +10937,11 @@
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr"/>
-      <c r="E109" s="11" t="inlineStr"/>
+      <c r="E109" s="11" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
       <c r="F109" s="11" t="inlineStr"/>
       <c r="G109" s="11" t="inlineStr">
         <is>
@@ -10731,7 +11025,11 @@
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr"/>
-      <c r="E110" s="5" t="inlineStr"/>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>291</t>
+        </is>
+      </c>
       <c r="F110" s="5" t="inlineStr"/>
       <c r="G110" s="5" t="inlineStr">
         <is>
@@ -10815,7 +11113,11 @@
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr"/>
-      <c r="E111" s="11" t="inlineStr"/>
+      <c r="E111" s="11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="F111" s="11" t="inlineStr"/>
       <c r="G111" s="11" t="inlineStr">
         <is>
@@ -10899,7 +11201,11 @@
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr"/>
-      <c r="E112" s="5" t="inlineStr"/>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
       <c r="F112" s="5" t="inlineStr"/>
       <c r="G112" s="5" t="inlineStr">
         <is>
@@ -10985,7 +11291,7 @@
       <c r="D113" s="10" t="inlineStr"/>
       <c r="E113" s="11" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>67</t>
         </is>
       </c>
       <c r="F113" s="11" t="inlineStr">
@@ -11060,7 +11366,7 @@
       </c>
       <c r="T113" s="11" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>+998 70 518-05-60 / +998 99 730-77-09 (Onasi)</t>
         </is>
       </c>
       <c r="U113" s="7" t="inlineStr">
@@ -11095,7 +11401,11 @@
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr"/>
-      <c r="E114" s="5" t="inlineStr"/>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
       <c r="F114" s="5" t="inlineStr"/>
       <c r="G114" s="5" t="inlineStr">
         <is>
@@ -11181,7 +11491,7 @@
       <c r="D115" s="10" t="inlineStr"/>
       <c r="E115" s="11" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>81</t>
         </is>
       </c>
       <c r="F115" s="18" t="n">
@@ -11250,7 +11560,7 @@
       </c>
       <c r="T115" s="11" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>+998 99 153-48-38 / +998 70 034-22-44 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U115" s="7" t="inlineStr">
@@ -11285,7 +11595,11 @@
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr"/>
-      <c r="E116" s="5" t="inlineStr"/>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>271</t>
+        </is>
+      </c>
       <c r="F116" s="5" t="inlineStr"/>
       <c r="G116" s="5" t="inlineStr">
         <is>
@@ -11375,7 +11689,7 @@
       </c>
       <c r="E117" s="11" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>254</t>
         </is>
       </c>
       <c r="F117" s="11" t="inlineStr">
@@ -11450,7 +11764,7 @@
       </c>
       <c r="T117" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 005-29-65 / +998 87 486-12-08 (Onasi)</t>
         </is>
       </c>
       <c r="U117" s="7" t="inlineStr">
@@ -11491,7 +11805,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F118" s="5" t="inlineStr">
@@ -11562,7 +11876,7 @@
       </c>
       <c r="T118" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 76 294-50-80 / +998 87 381-98-20 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U118" s="7" t="inlineStr">
@@ -11603,7 +11917,7 @@
       <c r="D119" s="10" t="inlineStr"/>
       <c r="E119" s="11" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>74</t>
         </is>
       </c>
       <c r="F119" s="11" t="inlineStr">
@@ -11666,7 +11980,7 @@
       </c>
       <c r="T119" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 587-79-09</t>
         </is>
       </c>
       <c r="U119" s="17" t="inlineStr">
@@ -11701,7 +12015,11 @@
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr"/>
-      <c r="E120" s="5" t="inlineStr"/>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="F120" s="5" t="inlineStr"/>
       <c r="G120" s="5" t="inlineStr">
         <is>
@@ -11795,7 +12113,7 @@
       </c>
       <c r="E121" s="11" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F121" s="18" t="n">
@@ -11868,7 +12186,7 @@
       </c>
       <c r="T121" s="11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 88 388-93-26 / +998 99 685-13-21 (O'zi)</t>
         </is>
       </c>
       <c r="U121" s="7" t="inlineStr">
@@ -11905,7 +12223,7 @@
       <c r="D122" s="4" t="inlineStr"/>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>263</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
@@ -11980,7 +12298,7 @@
       </c>
       <c r="T122" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 010-26-21 / +998 97 701-17-83 (Onasi)</t>
         </is>
       </c>
       <c r="U122" s="7" t="inlineStr">
@@ -12021,7 +12339,7 @@
       </c>
       <c r="E123" s="11" t="inlineStr">
         <is>
-          <t>275</t>
+          <t>107</t>
         </is>
       </c>
       <c r="F123" s="11" t="inlineStr">
@@ -12096,7 +12414,7 @@
       </c>
       <c r="T123" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 005-49-08 / +998 93 553-33-51 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U123" s="7" t="inlineStr">
@@ -12141,7 +12459,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>57</t>
         </is>
       </c>
       <c r="F124" s="5" t="inlineStr">
@@ -12208,7 +12526,7 @@
       </c>
       <c r="T124" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 568-15-08 / +998 88 585-70-68 (Otasi)</t>
         </is>
       </c>
       <c r="U124" s="15" t="inlineStr">
@@ -12243,7 +12561,11 @@
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr"/>
-      <c r="E125" s="11" t="inlineStr"/>
+      <c r="E125" s="11" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
       <c r="F125" s="11" t="inlineStr"/>
       <c r="G125" s="11" t="inlineStr">
         <is>
@@ -12307,7 +12629,11 @@
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr"/>
-      <c r="E126" s="5" t="inlineStr"/>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>172</t>
+        </is>
+      </c>
       <c r="F126" s="5" t="inlineStr"/>
       <c r="G126" s="5" t="inlineStr">
         <is>
@@ -12389,7 +12715,7 @@
       <c r="D127" s="10" t="inlineStr"/>
       <c r="E127" s="11" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>288</t>
         </is>
       </c>
       <c r="F127" s="11" t="inlineStr">
@@ -12464,7 +12790,7 @@
       </c>
       <c r="T127" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 335-05-82 / +998 97 863-50-82 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U127" s="7" t="inlineStr">
@@ -12503,7 +12829,11 @@
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr"/>
-      <c r="E128" s="5" t="inlineStr"/>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>306</t>
+        </is>
+      </c>
       <c r="F128" s="5" t="inlineStr"/>
       <c r="G128" s="5" t="inlineStr">
         <is>
@@ -12587,7 +12917,11 @@
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr"/>
-      <c r="E129" s="11" t="inlineStr"/>
+      <c r="E129" s="11" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
       <c r="F129" s="11" t="inlineStr"/>
       <c r="G129" s="11" t="inlineStr">
         <is>
@@ -12685,7 +13019,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F130" s="5" t="inlineStr">
@@ -12760,7 +13094,7 @@
       </c>
       <c r="T130" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 91 217-70-09 / +998 91 460-65-62 (Akasi)</t>
         </is>
       </c>
       <c r="U130" s="7" t="inlineStr">
@@ -12795,7 +13129,11 @@
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr"/>
-      <c r="E131" s="11" t="inlineStr"/>
+      <c r="E131" s="11" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
       <c r="F131" s="11" t="inlineStr"/>
       <c r="G131" s="11" t="inlineStr">
         <is>
@@ -12879,7 +13217,11 @@
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr"/>
-      <c r="E132" s="5" t="inlineStr"/>
+      <c r="E132" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="F132" s="5" t="inlineStr"/>
       <c r="G132" s="5" t="inlineStr">
         <is>
@@ -12963,7 +13305,11 @@
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr"/>
-      <c r="E133" s="11" t="inlineStr"/>
+      <c r="E133" s="11" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="F133" s="11" t="inlineStr"/>
       <c r="G133" s="11" t="inlineStr">
         <is>
@@ -13053,7 +13399,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>388</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
@@ -13124,7 +13470,7 @@
       </c>
       <c r="T134" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 495-26-08 / +998 97 387-38-03 (Onasi)</t>
         </is>
       </c>
       <c r="U134" s="17" t="inlineStr">
@@ -13159,7 +13505,11 @@
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr"/>
-      <c r="E135" s="11" t="inlineStr"/>
+      <c r="E135" s="11" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
       <c r="F135" s="11" t="inlineStr"/>
       <c r="G135" s="11" t="inlineStr">
         <is>
@@ -13239,7 +13589,11 @@
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr"/>
-      <c r="E136" s="5" t="inlineStr"/>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
       <c r="F136" s="5" t="inlineStr"/>
       <c r="G136" s="5" t="inlineStr">
         <is>
@@ -13319,7 +13673,11 @@
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr"/>
-      <c r="E137" s="11" t="inlineStr"/>
+      <c r="E137" s="11" t="inlineStr">
+        <is>
+          <t>268</t>
+        </is>
+      </c>
       <c r="F137" s="11" t="inlineStr"/>
       <c r="G137" s="11" t="inlineStr">
         <is>
@@ -13405,7 +13763,7 @@
       <c r="D138" s="4" t="inlineStr"/>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F138" s="12" t="n">
@@ -13478,7 +13836,7 @@
       </c>
       <c r="T138" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 95 259-06-25 / +998 99 152-33-71 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U138" s="7" t="inlineStr">
@@ -13513,7 +13871,11 @@
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr"/>
-      <c r="E139" s="11" t="inlineStr"/>
+      <c r="E139" s="11" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
       <c r="F139" s="11" t="inlineStr"/>
       <c r="G139" s="11" t="inlineStr">
         <is>
@@ -13597,7 +13959,11 @@
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr"/>
-      <c r="E140" s="5" t="inlineStr"/>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
       <c r="F140" s="5" t="inlineStr"/>
       <c r="G140" s="5" t="inlineStr">
         <is>
@@ -13681,7 +14047,11 @@
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr"/>
-      <c r="E141" s="11" t="inlineStr"/>
+      <c r="E141" s="11" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
       <c r="F141" s="11" t="inlineStr"/>
       <c r="G141" s="11" t="inlineStr">
         <is>
@@ -13765,7 +14135,11 @@
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr"/>
-      <c r="E142" s="5" t="inlineStr"/>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
       <c r="F142" s="5" t="inlineStr"/>
       <c r="G142" s="5" t="inlineStr">
         <is>
@@ -13849,7 +14223,11 @@
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr"/>
-      <c r="E143" s="11" t="inlineStr"/>
+      <c r="E143" s="11" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
       <c r="F143" s="11" t="inlineStr"/>
       <c r="G143" s="11" t="inlineStr">
         <is>
@@ -13939,7 +14317,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>294</t>
+          <t>280</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
@@ -14010,7 +14388,7 @@
       </c>
       <c r="T144" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 115-10-31 / +998 88 184-05-85 (Onasi)</t>
         </is>
       </c>
       <c r="U144" s="7" t="inlineStr">
@@ -14053,7 +14431,11 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E145" s="11" t="inlineStr"/>
+      <c r="E145" s="11" t="inlineStr">
+        <is>
+          <t>313</t>
+        </is>
+      </c>
       <c r="F145" s="11" t="inlineStr"/>
       <c r="G145" s="11" t="inlineStr">
         <is>
@@ -14145,7 +14527,11 @@
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr"/>
-      <c r="E146" s="5" t="inlineStr"/>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
       <c r="F146" s="5" t="inlineStr"/>
       <c r="G146" s="5" t="inlineStr">
         <is>
@@ -14229,7 +14615,11 @@
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr"/>
-      <c r="E147" s="11" t="inlineStr"/>
+      <c r="E147" s="11" t="inlineStr">
+        <is>
+          <t>298</t>
+        </is>
+      </c>
       <c r="F147" s="11" t="inlineStr"/>
       <c r="G147" s="11" t="inlineStr">
         <is>
@@ -14315,7 +14705,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>148</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
@@ -14388,11 +14778,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T148" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T148" s="5" t="inlineStr"/>
       <c r="U148" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -14425,7 +14811,11 @@
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr"/>
-      <c r="E149" s="11" t="inlineStr"/>
+      <c r="E149" s="11" t="inlineStr">
+        <is>
+          <t>279</t>
+        </is>
+      </c>
       <c r="F149" s="11" t="inlineStr"/>
       <c r="G149" s="11" t="inlineStr">
         <is>
@@ -14509,7 +14899,11 @@
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr"/>
-      <c r="E150" s="5" t="inlineStr"/>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>283</t>
+        </is>
+      </c>
       <c r="F150" s="5" t="inlineStr"/>
       <c r="G150" s="5" t="inlineStr">
         <is>
@@ -14599,7 +14993,7 @@
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>188</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
@@ -14670,7 +15064,7 @@
       </c>
       <c r="T151" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 83 403-00-80 / +998 95 264-70-90 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U151" s="7" t="inlineStr">
@@ -14709,7 +15103,11 @@
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr"/>
-      <c r="E152" s="5" t="inlineStr"/>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
       <c r="F152" s="5" t="inlineStr"/>
       <c r="G152" s="5" t="inlineStr">
         <is>
@@ -14799,7 +15197,7 @@
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr"/>
@@ -14866,7 +15264,7 @@
       </c>
       <c r="T153" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 81 831-16-70 / +998 18 311-67-87 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U153" s="7" t="inlineStr">
@@ -14911,7 +15309,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>181</t>
         </is>
       </c>
       <c r="F154" s="5" t="inlineStr"/>
@@ -14974,7 +15372,7 @@
       </c>
       <c r="T154" s="5" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>+998 87 358-87-97 / +998 88 632-19-72 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U154" s="5" t="inlineStr"/>
@@ -15001,7 +15399,11 @@
         </is>
       </c>
       <c r="D155" s="10" t="inlineStr"/>
-      <c r="E155" s="11" t="inlineStr"/>
+      <c r="E155" s="11" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
       <c r="F155" s="11" t="inlineStr"/>
       <c r="G155" s="11" t="inlineStr">
         <is>
@@ -15091,7 +15493,7 @@
       </c>
       <c r="E156" s="5" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>116</t>
         </is>
       </c>
       <c r="F156" s="5" t="inlineStr">
@@ -15166,7 +15568,7 @@
       </c>
       <c r="T156" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 79 347-60-80 / +998 91 456-46-61 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U156" s="7" t="inlineStr">
@@ -15201,7 +15603,11 @@
         </is>
       </c>
       <c r="D157" s="10" t="inlineStr"/>
-      <c r="E157" s="11" t="inlineStr"/>
+      <c r="E157" s="11" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
       <c r="F157" s="11" t="inlineStr"/>
       <c r="G157" s="11" t="inlineStr">
         <is>
@@ -15281,7 +15687,11 @@
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr"/>
-      <c r="E158" s="5" t="inlineStr"/>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
       <c r="F158" s="5" t="inlineStr"/>
       <c r="G158" s="5" t="inlineStr">
         <is>
@@ -15365,7 +15775,11 @@
         </is>
       </c>
       <c r="D159" s="10" t="inlineStr"/>
-      <c r="E159" s="11" t="inlineStr"/>
+      <c r="E159" s="11" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
       <c r="F159" s="11" t="inlineStr"/>
       <c r="G159" s="11" t="inlineStr">
         <is>
@@ -15455,7 +15869,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>307</t>
         </is>
       </c>
       <c r="F160" s="5" t="inlineStr">
@@ -15530,7 +15944,7 @@
       </c>
       <c r="T160" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 618-02-59</t>
         </is>
       </c>
       <c r="U160" s="7" t="inlineStr">
@@ -15565,7 +15979,11 @@
         </is>
       </c>
       <c r="D161" s="10" t="inlineStr"/>
-      <c r="E161" s="11" t="inlineStr"/>
+      <c r="E161" s="11" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
       <c r="F161" s="11" t="inlineStr"/>
       <c r="G161" s="11" t="inlineStr">
         <is>
@@ -15655,7 +16073,7 @@
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>232</t>
         </is>
       </c>
       <c r="F162" s="5" t="inlineStr">
@@ -15730,7 +16148,7 @@
       </c>
       <c r="T162" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 952-43-44 / +998 90 442-22-47 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U162" s="7" t="inlineStr">
@@ -15771,7 +16189,7 @@
       </c>
       <c r="E163" s="11" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>234</t>
         </is>
       </c>
       <c r="F163" s="11" t="inlineStr">
@@ -15834,7 +16252,7 @@
       </c>
       <c r="T163" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 00 111-40-90 / +998 97 389-11-74 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U163" s="17" t="inlineStr">
@@ -15875,7 +16293,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t>262</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F164" s="5" t="inlineStr">
@@ -15950,7 +16368,7 @@
       </c>
       <c r="T164" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 811-22-08 / +998 91 815-13-09 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U164" s="7" t="inlineStr">
@@ -15985,7 +16403,11 @@
         </is>
       </c>
       <c r="D165" s="10" t="inlineStr"/>
-      <c r="E165" s="11" t="inlineStr"/>
+      <c r="E165" s="11" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
       <c r="F165" s="11" t="inlineStr"/>
       <c r="G165" s="11" t="inlineStr">
         <is>
@@ -16075,7 +16497,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F166" s="5" t="inlineStr">
@@ -16150,7 +16572,7 @@
       </c>
       <c r="T166" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 80 880-12-40 / +998 15 613-00-20 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U166" s="7" t="inlineStr">
@@ -16185,7 +16607,11 @@
         </is>
       </c>
       <c r="D167" s="10" t="inlineStr"/>
-      <c r="E167" s="11" t="inlineStr"/>
+      <c r="E167" s="11" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
       <c r="F167" s="11" t="inlineStr"/>
       <c r="G167" s="11" t="inlineStr">
         <is>
@@ -16269,7 +16695,11 @@
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr"/>
-      <c r="E168" s="5" t="inlineStr"/>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
       <c r="F168" s="5" t="inlineStr"/>
       <c r="G168" s="5" t="inlineStr">
         <is>
@@ -16349,7 +16779,11 @@
         </is>
       </c>
       <c r="D169" s="10" t="inlineStr"/>
-      <c r="E169" s="11" t="inlineStr"/>
+      <c r="E169" s="11" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
       <c r="F169" s="11" t="inlineStr"/>
       <c r="G169" s="11" t="inlineStr">
         <is>
@@ -16433,7 +16867,11 @@
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr"/>
-      <c r="E170" s="5" t="inlineStr"/>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
       <c r="F170" s="5" t="inlineStr"/>
       <c r="G170" s="5" t="inlineStr">
         <is>
@@ -16517,7 +16955,11 @@
         </is>
       </c>
       <c r="D171" s="10" t="inlineStr"/>
-      <c r="E171" s="11" t="inlineStr"/>
+      <c r="E171" s="11" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
       <c r="F171" s="11" t="inlineStr"/>
       <c r="G171" s="11" t="inlineStr">
         <is>
@@ -16607,7 +17049,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>387</t>
         </is>
       </c>
       <c r="F172" s="5" t="inlineStr">
@@ -16682,7 +17124,7 @@
       </c>
       <c r="T172" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 50 202-81-30 / +998 72 752-81-30 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U172" s="7" t="inlineStr">
@@ -16723,7 +17165,7 @@
       </c>
       <c r="E173" s="11" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>233</t>
         </is>
       </c>
       <c r="F173" s="11" t="inlineStr">
@@ -16794,7 +17236,7 @@
       </c>
       <c r="T173" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 97 852-74-04 / +998 97 852-74-04 (O'zi)</t>
         </is>
       </c>
       <c r="U173" s="7" t="inlineStr">
@@ -16833,7 +17275,11 @@
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr"/>
-      <c r="E174" s="5" t="inlineStr"/>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
       <c r="F174" s="5" t="inlineStr"/>
       <c r="G174" s="5" t="inlineStr">
         <is>
@@ -16921,7 +17367,11 @@
         </is>
       </c>
       <c r="D175" s="10" t="inlineStr"/>
-      <c r="E175" s="11" t="inlineStr"/>
+      <c r="E175" s="11" t="inlineStr">
+        <is>
+          <t>273</t>
+        </is>
+      </c>
       <c r="F175" s="11" t="inlineStr"/>
       <c r="G175" s="11" t="inlineStr">
         <is>
@@ -16987,7 +17437,7 @@
       <c r="D176" s="4" t="inlineStr"/>
       <c r="E176" s="5" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>318</t>
         </is>
       </c>
       <c r="F176" s="5" t="inlineStr">
@@ -17058,7 +17508,7 @@
       </c>
       <c r="T176" s="5" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>+998 59 399-20-50 / +998 52 332-76-60 (Qaynonasi)</t>
         </is>
       </c>
       <c r="U176" s="7" t="inlineStr">
@@ -17256,11 +17706,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T178" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
+      <c r="T178" s="5" t="inlineStr"/>
       <c r="U178" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -17297,7 +17743,11 @@
         </is>
       </c>
       <c r="D179" s="10" t="inlineStr"/>
-      <c r="E179" s="11" t="inlineStr"/>
+      <c r="E179" s="11" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="F179" s="11" t="inlineStr"/>
       <c r="G179" s="11" t="inlineStr">
         <is>
@@ -17633,7 +18083,11 @@
         </is>
       </c>
       <c r="D183" s="10" t="inlineStr"/>
-      <c r="E183" s="11" t="inlineStr"/>
+      <c r="E183" s="11" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
       <c r="F183" s="11" t="inlineStr"/>
       <c r="G183" s="11" t="inlineStr">
         <is>
@@ -17723,7 +18177,7 @@
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>326</t>
         </is>
       </c>
       <c r="F184" s="5" t="inlineStr">
@@ -17798,7 +18252,7 @@
       </c>
       <c r="T184" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 70 034-95-05 / +998 99 468-84-06 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U184" s="7" t="inlineStr">
@@ -17898,7 +18352,7 @@
       </c>
       <c r="T185" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 04 403-66-60 / +998 12 247-72-10 (Turmush o'rtog'i)</t>
         </is>
       </c>
       <c r="U185" s="17" t="inlineStr">
@@ -18342,7 +18796,7 @@
       </c>
       <c r="T190" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 70 120-65-08 / +998 99 569-81-12 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U190" s="7" t="inlineStr">
@@ -18538,7 +18992,7 @@
       </c>
       <c r="T192" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 99 673-99-29 / +998 99 673-99-29 (O'zi)</t>
         </is>
       </c>
       <c r="U192" s="7" t="inlineStr">
@@ -18646,7 +19100,7 @@
       </c>
       <c r="T193" s="11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 88 384-85-45</t>
         </is>
       </c>
       <c r="U193" s="11" t="inlineStr"/>
@@ -18836,7 +19290,7 @@
       </c>
       <c r="T195" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 90 815-25-00 / +998 94 817-01-93 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U195" s="7" t="inlineStr">
@@ -18952,7 +19406,7 @@
       </c>
       <c r="T196" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 33 296-07-08 / +998 88 136-09-26 (Onasi)</t>
         </is>
       </c>
       <c r="U196" s="7" t="inlineStr">
@@ -19208,7 +19662,7 @@
       </c>
       <c r="T199" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 91 810-81-91 / +998 90 099-57-63 (Onasi)</t>
         </is>
       </c>
       <c r="U199" s="7" t="inlineStr">
@@ -19660,7 +20114,7 @@
       </c>
       <c r="T204" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 732-61-11 / +998 90 617-68-83 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U204" s="7" t="inlineStr">
@@ -19766,7 +20220,7 @@
       <c r="S205" s="11" t="inlineStr"/>
       <c r="T205" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 04 504-24-00 / +998 93 903-47-44 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U205" s="15" t="inlineStr">
@@ -19958,7 +20412,7 @@
       </c>
       <c r="T207" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 217-14-30 / +998 94 134-34-03 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U207" s="7" t="inlineStr">
@@ -20074,7 +20528,7 @@
       </c>
       <c r="T208" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 18 440-30-80 / +998 19 594-21-50 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U208" s="7" t="inlineStr">
@@ -20272,8 +20726,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T210" s="5" t="n">
-        <v>2026</v>
+      <c r="T210" s="5" t="inlineStr">
+        <is>
+          <t>+998 91 464-92-28 / +998 88 601-52-00 (Onasi)</t>
+        </is>
       </c>
       <c r="U210" s="7" t="inlineStr">
         <is>
@@ -20472,7 +20928,7 @@
       </c>
       <c r="T212" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>+998 88 388-93-26 / +998 99 685-13-21 (O'zi)</t>
         </is>
       </c>
       <c r="U212" s="7" t="inlineStr">
@@ -20672,7 +21128,7 @@
       </c>
       <c r="T214" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 72 130-24-00 / +998 86 188-58-00 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U214" s="7" t="inlineStr">
@@ -21362,7 +21818,7 @@
       </c>
       <c r="T222" s="5" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>+998 16 354-55-60 / +998 95 333-29-60 (Turmush o'rtog'i)</t>
         </is>
       </c>
       <c r="U222" s="7" t="inlineStr">
@@ -21714,7 +22170,7 @@
       </c>
       <c r="T226" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 716-01-30 / +998 88 388-79-12 (Onasi)</t>
         </is>
       </c>
       <c r="U226" s="7" t="inlineStr">
@@ -22078,7 +22534,7 @@
       </c>
       <c r="T230" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 217-70-09 / +998 91 460-65-62 (Akasi)</t>
         </is>
       </c>
       <c r="U230" s="7" t="inlineStr">
@@ -22278,7 +22734,7 @@
       </c>
       <c r="T232" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 463-79-08 / +998 10 709-57-90 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U232" s="7" t="inlineStr">
@@ -22388,11 +22844,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T233" s="11" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
+      <c r="T233" s="11" t="inlineStr"/>
       <c r="U233" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -22683,7 +23135,7 @@
       </c>
       <c r="E237" s="11" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26/27 Sh/A 268</t>
         </is>
       </c>
       <c r="F237" s="11" t="inlineStr">
@@ -22752,8 +23204,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T237" s="11" t="n">
-        <v>2009</v>
+      <c r="T237" s="11" t="inlineStr">
+        <is>
+          <t>+998 88 803-91-93 / +998 88 726-14-12 (Otasi / Onasi)</t>
+        </is>
       </c>
       <c r="U237" s="7" t="inlineStr">
         <is>
@@ -22793,7 +23247,7 @@
       <c r="D238" s="4" t="inlineStr"/>
       <c r="E238" s="5" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>26/27 SH/A 216</t>
         </is>
       </c>
       <c r="F238" s="5" t="inlineStr">
@@ -22862,11 +23316,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T238" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T238" s="5" t="inlineStr"/>
       <c r="U238" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -22905,7 +23355,7 @@
       <c r="D239" s="10" t="inlineStr"/>
       <c r="E239" s="11" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>26/27 SH/A 33</t>
         </is>
       </c>
       <c r="F239" s="18" t="n">
@@ -22974,7 +23424,7 @@
       </c>
       <c r="T239" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 88 399-00-96</t>
         </is>
       </c>
       <c r="U239" s="7" t="inlineStr">
@@ -23013,7 +23463,11 @@
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr"/>
-      <c r="E240" s="5" t="inlineStr"/>
+      <c r="E240" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A269</t>
+        </is>
+      </c>
       <c r="F240" s="5" t="inlineStr"/>
       <c r="G240" s="5" t="inlineStr">
         <is>
@@ -23338,7 +23792,7 @@
       </c>
       <c r="T243" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 76 590-02-70 / +998 70 790-86-80 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U243" s="7" t="inlineStr">
@@ -23459,7 +23913,7 @@
       <c r="D245" s="10" t="inlineStr"/>
       <c r="E245" s="11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>25/26 sh/a 6</t>
         </is>
       </c>
       <c r="F245" s="18" t="n">
@@ -23528,7 +23982,7 @@
       </c>
       <c r="T245" s="11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 70 188-54-32 / +998 95 805-01-86 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U245" s="7" t="inlineStr">
@@ -23806,7 +24260,7 @@
       </c>
       <c r="T248" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 625-99-07</t>
         </is>
       </c>
       <c r="U248" s="7" t="inlineStr">
@@ -24000,11 +24454,7 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="T250" s="5" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
+      <c r="T250" s="5" t="inlineStr"/>
       <c r="U250" s="5" t="inlineStr">
         <is>
           <t>To'liq</t>
@@ -24105,7 +24555,11 @@
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr"/>
-      <c r="E252" s="5" t="inlineStr"/>
+      <c r="E252" s="5" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 33</t>
+        </is>
+      </c>
       <c r="F252" s="5" t="inlineStr"/>
       <c r="G252" s="5" t="inlineStr">
         <is>
@@ -24189,7 +24643,11 @@
         </is>
       </c>
       <c r="D253" s="10" t="inlineStr"/>
-      <c r="E253" s="11" t="inlineStr"/>
+      <c r="E253" s="11" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A 220</t>
+        </is>
+      </c>
       <c r="F253" s="11" t="inlineStr"/>
       <c r="G253" s="11" t="inlineStr">
         <is>
@@ -24273,7 +24731,11 @@
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr"/>
-      <c r="E254" s="5" t="inlineStr"/>
+      <c r="E254" s="5" t="inlineStr">
+        <is>
+          <t>26/27 sh/a 277</t>
+        </is>
+      </c>
       <c r="F254" s="5" t="inlineStr"/>
       <c r="G254" s="5" t="inlineStr">
         <is>
@@ -24443,7 +24905,7 @@
       <c r="D256" s="4" t="inlineStr"/>
       <c r="E256" s="5" t="inlineStr">
         <is>
-          <t>258</t>
+          <t>25/26 SH/A57</t>
         </is>
       </c>
       <c r="F256" s="5" t="inlineStr">
@@ -24506,7 +24968,7 @@
       <c r="S256" s="5" t="inlineStr"/>
       <c r="T256" s="5" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>+998 91 957-18-58</t>
         </is>
       </c>
       <c r="U256" s="15" t="inlineStr">
@@ -25490,7 +25952,7 @@
       </c>
       <c r="T267" s="11" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>+998 73 865-61-20 / +998 73 824-60-60 (Turmush o'rtog'i)</t>
         </is>
       </c>
       <c r="U267" s="17" t="inlineStr">
@@ -25778,7 +26240,7 @@
       </c>
       <c r="T270" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 800-66-37 / +998 97 001-27-80 (Onasi)</t>
         </is>
       </c>
       <c r="U270" s="7" t="inlineStr">
@@ -25813,7 +26275,11 @@
         </is>
       </c>
       <c r="D271" s="10" t="inlineStr"/>
-      <c r="E271" s="11" t="inlineStr"/>
+      <c r="E271" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 226</t>
+        </is>
+      </c>
       <c r="F271" s="11" t="inlineStr"/>
       <c r="G271" s="11" t="inlineStr">
         <is>
@@ -25981,7 +26447,11 @@
         </is>
       </c>
       <c r="D273" s="10" t="inlineStr"/>
-      <c r="E273" s="11" t="inlineStr"/>
+      <c r="E273" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A252</t>
+        </is>
+      </c>
       <c r="F273" s="11" t="inlineStr"/>
       <c r="G273" s="11" t="inlineStr">
         <is>
@@ -26045,7 +26515,11 @@
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr"/>
-      <c r="E274" s="5" t="inlineStr"/>
+      <c r="E274" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 285</t>
+        </is>
+      </c>
       <c r="F274" s="5" t="inlineStr"/>
       <c r="G274" s="5" t="inlineStr">
         <is>
@@ -26129,7 +26603,11 @@
         </is>
       </c>
       <c r="D275" s="10" t="inlineStr"/>
-      <c r="E275" s="11" t="inlineStr"/>
+      <c r="E275" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 285</t>
+        </is>
+      </c>
       <c r="F275" s="11" t="inlineStr"/>
       <c r="G275" s="11" t="inlineStr">
         <is>
@@ -26284,11 +26762,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T276" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T276" s="5" t="inlineStr"/>
       <c r="U276" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -26321,7 +26795,11 @@
         </is>
       </c>
       <c r="D277" s="10" t="inlineStr"/>
-      <c r="E277" s="11" t="inlineStr"/>
+      <c r="E277" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 286</t>
+        </is>
+      </c>
       <c r="F277" s="11" t="inlineStr"/>
       <c r="G277" s="11" t="inlineStr">
         <is>
@@ -27050,7 +27528,7 @@
       </c>
       <c r="T285" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 99 819-11-07</t>
         </is>
       </c>
       <c r="U285" s="7" t="inlineStr">
@@ -27166,7 +27644,7 @@
       </c>
       <c r="T286" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 77 607-08-24 / +998 73 990-17-90 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U286" s="7" t="inlineStr">
@@ -27260,11 +27738,7 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T287" s="11" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
+      <c r="T287" s="11" t="inlineStr"/>
       <c r="U287" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -27372,11 +27846,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T288" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T288" s="5" t="inlineStr"/>
       <c r="U288" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -27419,7 +27889,7 @@
       </c>
       <c r="E289" s="11" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>26/27 SH/A 288</t>
         </is>
       </c>
       <c r="F289" s="11" t="inlineStr">
@@ -27494,7 +27964,7 @@
       </c>
       <c r="T289" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 70 108-08-29 / +998 99 246-08-29 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U289" s="7" t="inlineStr">
@@ -27789,7 +28259,11 @@
         </is>
       </c>
       <c r="D293" s="10" t="inlineStr"/>
-      <c r="E293" s="11" t="inlineStr"/>
+      <c r="E293" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 259</t>
+        </is>
+      </c>
       <c r="F293" s="11" t="inlineStr"/>
       <c r="G293" s="11" t="inlineStr">
         <is>
@@ -27873,7 +28347,11 @@
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr"/>
-      <c r="E294" s="5" t="inlineStr"/>
+      <c r="E294" s="5" t="inlineStr">
+        <is>
+          <t>26/27 sh/a 235</t>
+        </is>
+      </c>
       <c r="F294" s="5" t="inlineStr"/>
       <c r="G294" s="5" t="inlineStr">
         <is>
@@ -28198,7 +28676,7 @@
       </c>
       <c r="T297" s="11" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>+998 91 949-16-27 / +998 90 069-89-98 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U297" s="7" t="inlineStr">
@@ -28449,7 +28927,11 @@
         </is>
       </c>
       <c r="D301" s="10" t="inlineStr"/>
-      <c r="E301" s="11" t="inlineStr"/>
+      <c r="E301" s="11" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A 239</t>
+        </is>
+      </c>
       <c r="F301" s="11" t="inlineStr"/>
       <c r="G301" s="11" t="inlineStr">
         <is>
@@ -28533,7 +29015,11 @@
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr"/>
-      <c r="E302" s="5" t="inlineStr"/>
+      <c r="E302" s="5" t="inlineStr">
+        <is>
+          <t>24/25 SH/A 41</t>
+        </is>
+      </c>
       <c r="F302" s="5" t="inlineStr">
         <is>
           <t>2026-09-08 00:00:00</t>
@@ -28887,7 +29373,7 @@
       </c>
       <c r="E306" s="5" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>26/27 SH/A 241</t>
         </is>
       </c>
       <c r="F306" s="5" t="inlineStr">
@@ -28958,7 +29444,7 @@
       </c>
       <c r="T306" s="5" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>+998 88 829-82-80 / +998 88 303-82-80 (Turmush o'rtog'i)</t>
         </is>
       </c>
       <c r="U306" s="7" t="inlineStr">
@@ -29216,7 +29702,7 @@
       </c>
       <c r="T309" s="11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 99 106-08-10 / +998 95 527-81-80 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U309" s="7" t="inlineStr">
@@ -29414,11 +29900,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T311" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T311" s="11" t="inlineStr"/>
       <c r="U311" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -29457,7 +29939,7 @@
       </c>
       <c r="E312" s="5" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>25/26 SH/A 286</t>
         </is>
       </c>
       <c r="F312" s="5" t="inlineStr">
@@ -29532,7 +30014,7 @@
       </c>
       <c r="T312" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 90 453-21-25</t>
         </is>
       </c>
       <c r="U312" s="7" t="inlineStr">
@@ -29819,7 +30301,11 @@
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr"/>
-      <c r="E316" s="5" t="inlineStr"/>
+      <c r="E316" s="5" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 506</t>
+        </is>
+      </c>
       <c r="F316" s="5" t="inlineStr"/>
       <c r="G316" s="5" t="inlineStr">
         <is>
@@ -29980,7 +30466,7 @@
       </c>
       <c r="T317" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 90 884-12-08 / +998 91 957-27-17 (Akasi)</t>
         </is>
       </c>
       <c r="U317" s="7" t="inlineStr">
@@ -30105,7 +30591,7 @@
       </c>
       <c r="E319" s="11" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>25/26 Sh/A509</t>
         </is>
       </c>
       <c r="F319" s="11" t="inlineStr">
@@ -30172,7 +30658,7 @@
       </c>
       <c r="T319" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 87 392-00-25 / +998 87 392-00-21 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U319" s="17" t="inlineStr">
@@ -30540,7 +31026,7 @@
       </c>
       <c r="T323" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 93 356-50-22 / +998 91 090-16-27 (Onasi)</t>
         </is>
       </c>
       <c r="U323" s="7" t="inlineStr">
@@ -30904,7 +31390,7 @@
       </c>
       <c r="T327" s="11" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>+998 88 387-94-04 / +998 88 381-39-79 (Onasi)</t>
         </is>
       </c>
       <c r="U327" s="15" t="inlineStr">
@@ -31096,7 +31582,7 @@
       </c>
       <c r="T329" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 632-37-73 / +998 91 470-84-93 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U329" s="15" t="inlineStr">
@@ -31135,7 +31621,11 @@
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr"/>
-      <c r="E330" s="5" t="inlineStr"/>
+      <c r="E330" s="5" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 520</t>
+        </is>
+      </c>
       <c r="F330" s="5" t="inlineStr"/>
       <c r="G330" s="5" t="inlineStr">
         <is>
@@ -31567,7 +32057,11 @@
         </is>
       </c>
       <c r="D335" s="10" t="inlineStr"/>
-      <c r="E335" s="11" t="inlineStr"/>
+      <c r="E335" s="11" t="inlineStr">
+        <is>
+          <t>25/26 sh/a 186</t>
+        </is>
+      </c>
       <c r="F335" s="11" t="inlineStr"/>
       <c r="G335" s="11" t="inlineStr">
         <is>
@@ -31735,7 +32229,11 @@
         </is>
       </c>
       <c r="D337" s="10" t="inlineStr"/>
-      <c r="E337" s="11" t="inlineStr"/>
+      <c r="E337" s="11" t="inlineStr">
+        <is>
+          <t>25/26 Sh/A 116</t>
+        </is>
+      </c>
       <c r="F337" s="11" t="inlineStr"/>
       <c r="G337" s="11" t="inlineStr">
         <is>
@@ -31984,7 +32482,7 @@
       </c>
       <c r="T339" s="11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 08 785-10-50 / +998 16 397-68-50 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U339" s="7" t="inlineStr">
@@ -32695,7 +33193,11 @@
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr"/>
-      <c r="E348" s="5" t="inlineStr"/>
+      <c r="E348" s="5" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A 327</t>
+        </is>
+      </c>
       <c r="F348" s="5" t="inlineStr"/>
       <c r="G348" s="5" t="inlineStr">
         <is>
@@ -33124,7 +33626,7 @@
       </c>
       <c r="T352" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>+998 50 158-27-29 / +998 99 730-48-04 (Onasi)</t>
         </is>
       </c>
       <c r="U352" s="7" t="inlineStr">
@@ -33406,11 +33908,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T355" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T355" s="11" t="inlineStr"/>
       <c r="U355" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -33848,7 +34346,7 @@
       </c>
       <c r="T360" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 387-28-25 / +998 91 218-44-36 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U360" s="17" t="inlineStr">
@@ -34044,7 +34542,7 @@
       </c>
       <c r="T362" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 90 677-80-76</t>
         </is>
       </c>
       <c r="U362" s="7" t="inlineStr">
@@ -34083,7 +34581,11 @@
         </is>
       </c>
       <c r="D363" s="10" t="inlineStr"/>
-      <c r="E363" s="11" t="inlineStr"/>
+      <c r="E363" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 15</t>
+        </is>
+      </c>
       <c r="F363" s="11" t="inlineStr"/>
       <c r="G363" s="11" t="inlineStr">
         <is>
@@ -34238,8 +34740,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T364" s="5" t="n">
-        <v>2026</v>
+      <c r="T364" s="5" t="inlineStr">
+        <is>
+          <t>+998 88 063-26-08 / +998 97 336-01-40 (Otasi / Onasi)</t>
+        </is>
       </c>
       <c r="U364" s="7" t="inlineStr">
         <is>
@@ -34277,7 +34781,11 @@
         </is>
       </c>
       <c r="D365" s="10" t="inlineStr"/>
-      <c r="E365" s="11" t="inlineStr"/>
+      <c r="E365" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 10</t>
+        </is>
+      </c>
       <c r="F365" s="11" t="inlineStr"/>
       <c r="G365" s="11" t="inlineStr">
         <is>
@@ -34774,7 +35282,7 @@
       </c>
       <c r="T370" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 79 656-30-80 / +998 71 390-67-70 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U370" s="7" t="inlineStr">
@@ -34809,7 +35317,11 @@
         </is>
       </c>
       <c r="D371" s="10" t="inlineStr"/>
-      <c r="E371" s="11" t="inlineStr"/>
+      <c r="E371" s="11" t="inlineStr">
+        <is>
+          <t>25/26 SH/A84</t>
+        </is>
+      </c>
       <c r="F371" s="11" t="inlineStr"/>
       <c r="G371" s="11" t="inlineStr">
         <is>
@@ -35040,11 +35552,7 @@
         </is>
       </c>
       <c r="S373" s="11" t="inlineStr"/>
-      <c r="T373" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T373" s="11" t="inlineStr"/>
       <c r="U373" s="17" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -35245,7 +35753,11 @@
         </is>
       </c>
       <c r="D376" s="4" t="inlineStr"/>
-      <c r="E376" s="5" t="inlineStr"/>
+      <c r="E376" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 26</t>
+        </is>
+      </c>
       <c r="F376" s="5" t="inlineStr"/>
       <c r="G376" s="5" t="inlineStr">
         <is>
@@ -35413,7 +35925,11 @@
         </is>
       </c>
       <c r="D378" s="4" t="inlineStr"/>
-      <c r="E378" s="5" t="inlineStr"/>
+      <c r="E378" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 28</t>
+        </is>
+      </c>
       <c r="F378" s="5" t="inlineStr"/>
       <c r="G378" s="5" t="inlineStr">
         <is>
@@ -35574,7 +36090,7 @@
       </c>
       <c r="T379" s="11" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>+998 16 354-55-60 / +998 95 333-29-60 (Turmush o'rtog'i)</t>
         </is>
       </c>
       <c r="U379" s="7" t="inlineStr">
@@ -35615,7 +36131,7 @@
       </c>
       <c r="E380" s="5" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>25/26 Sh/A 107</t>
         </is>
       </c>
       <c r="F380" s="5" t="inlineStr"/>
@@ -35674,7 +36190,7 @@
       </c>
       <c r="T380" s="5" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>+998 91 219-20-99</t>
         </is>
       </c>
       <c r="U380" s="7" t="inlineStr">
@@ -35950,7 +36466,7 @@
       </c>
       <c r="T383" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 05 030-53-90 / +998 91 951-05-36 (Akasi)</t>
         </is>
       </c>
       <c r="U383" s="15" t="inlineStr">
@@ -36066,7 +36582,7 @@
       </c>
       <c r="T384" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 558-15-35 / +998 88 633-15-35 (Onasi)</t>
         </is>
       </c>
       <c r="U384" s="15" t="inlineStr">
@@ -36174,7 +36690,7 @@
       </c>
       <c r="T385" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 88 606-15-00 / +998 76 150-09-19 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U385" s="7" t="inlineStr">
@@ -36369,7 +36885,11 @@
         </is>
       </c>
       <c r="D388" s="4" t="inlineStr"/>
-      <c r="E388" s="5" t="inlineStr"/>
+      <c r="E388" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A40</t>
+        </is>
+      </c>
       <c r="F388" s="5" t="inlineStr"/>
       <c r="G388" s="5" t="inlineStr">
         <is>
@@ -36618,7 +37138,7 @@
       </c>
       <c r="T390" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 597-09-64</t>
         </is>
       </c>
       <c r="U390" s="7" t="inlineStr">
@@ -36922,7 +37442,7 @@
       </c>
       <c r="T393" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 31 522-57-70 / +998 77 086-77-25 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U393" s="7" t="inlineStr">
@@ -37206,7 +37726,7 @@
       </c>
       <c r="T396" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 000-14-58 / +998 90 517-61-63 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U396" s="7" t="inlineStr">
@@ -37325,7 +37845,11 @@
         </is>
       </c>
       <c r="D398" s="4" t="inlineStr"/>
-      <c r="E398" s="5" t="inlineStr"/>
+      <c r="E398" s="5" t="inlineStr">
+        <is>
+          <t>25/26 Sh/A 140</t>
+        </is>
+      </c>
       <c r="F398" s="5" t="inlineStr"/>
       <c r="G398" s="5" t="inlineStr">
         <is>
@@ -37411,7 +37935,7 @@
       <c r="D399" s="10" t="inlineStr"/>
       <c r="E399" s="11" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>25/26 SH/A149</t>
         </is>
       </c>
       <c r="F399" s="11" t="inlineStr">
@@ -37484,11 +38008,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T399" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T399" s="11" t="inlineStr"/>
       <c r="U399" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -37859,7 +38379,7 @@
       </c>
       <c r="E404" s="5" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>25/26 Sh/A 142</t>
         </is>
       </c>
       <c r="F404" s="5" t="inlineStr">
@@ -37934,7 +38454,7 @@
       </c>
       <c r="T404" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 94 082-51-16</t>
         </is>
       </c>
       <c r="U404" s="7" t="inlineStr">
@@ -37969,7 +38489,11 @@
         </is>
       </c>
       <c r="D405" s="10" t="inlineStr"/>
-      <c r="E405" s="11" t="inlineStr"/>
+      <c r="E405" s="11" t="inlineStr">
+        <is>
+          <t>25/26 SH/A150</t>
+        </is>
+      </c>
       <c r="F405" s="11" t="inlineStr"/>
       <c r="G405" s="11" t="inlineStr">
         <is>
@@ -38386,7 +38910,7 @@
       </c>
       <c r="T409" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 91 802-16-70 / +998 91 961-40-37 (Onasi)</t>
         </is>
       </c>
       <c r="U409" s="7" t="inlineStr">
@@ -38733,7 +39257,11 @@
         </is>
       </c>
       <c r="D414" s="4" t="inlineStr"/>
-      <c r="E414" s="5" t="inlineStr"/>
+      <c r="E414" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A66</t>
+        </is>
+      </c>
       <c r="F414" s="5" t="inlineStr"/>
       <c r="G414" s="5" t="inlineStr">
         <is>
@@ -39418,7 +39946,7 @@
       </c>
       <c r="T421" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 77 085-06-27 / +998 88 085-06-27 (Onasi)</t>
         </is>
       </c>
       <c r="U421" s="7" t="inlineStr">
@@ -39537,7 +40065,11 @@
         </is>
       </c>
       <c r="D423" s="10" t="inlineStr"/>
-      <c r="E423" s="11" t="inlineStr"/>
+      <c r="E423" s="11" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 74</t>
+        </is>
+      </c>
       <c r="F423" s="11" t="inlineStr"/>
       <c r="G423" s="11" t="inlineStr">
         <is>
@@ -39698,7 +40230,7 @@
       </c>
       <c r="T424" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 70 478-58-08 / +998 88 753-84-86 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U424" s="7" t="inlineStr">
@@ -39823,7 +40355,7 @@
       </c>
       <c r="E426" s="5" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>26/27 SH/A 76</t>
         </is>
       </c>
       <c r="F426" s="5" t="inlineStr">
@@ -39884,11 +40416,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T426" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
+      <c r="T426" s="5" t="inlineStr"/>
       <c r="U426" s="17" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -40009,7 +40537,11 @@
         </is>
       </c>
       <c r="D428" s="4" t="inlineStr"/>
-      <c r="E428" s="5" t="inlineStr"/>
+      <c r="E428" s="5" t="inlineStr">
+        <is>
+          <t>26/27 sh/a 78</t>
+        </is>
+      </c>
       <c r="F428" s="5" t="inlineStr"/>
       <c r="G428" s="5" t="inlineStr">
         <is>
@@ -40097,7 +40629,11 @@
         </is>
       </c>
       <c r="D429" s="10" t="inlineStr"/>
-      <c r="E429" s="11" t="inlineStr"/>
+      <c r="E429" s="11" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A79</t>
+        </is>
+      </c>
       <c r="F429" s="11" t="inlineStr"/>
       <c r="G429" s="11" t="inlineStr">
         <is>
@@ -40250,8 +40786,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T430" s="5" t="n">
-        <v>2026</v>
+      <c r="T430" s="5" t="inlineStr">
+        <is>
+          <t>+998 90 878-02-80 / +998 95 269-48-78 (Onasi)</t>
+        </is>
       </c>
       <c r="U430" s="7" t="inlineStr">
         <is>
@@ -40360,11 +40898,7 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="T431" s="11" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
+      <c r="T431" s="11" t="inlineStr"/>
       <c r="U431" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -40401,7 +40935,11 @@
         </is>
       </c>
       <c r="D432" s="4" t="inlineStr"/>
-      <c r="E432" s="5" t="inlineStr"/>
+      <c r="E432" s="5" t="inlineStr">
+        <is>
+          <t>25/26 sh/a 385</t>
+        </is>
+      </c>
       <c r="F432" s="5" t="inlineStr"/>
       <c r="G432" s="5" t="inlineStr">
         <is>
@@ -40677,7 +41215,11 @@
         </is>
       </c>
       <c r="D436" s="4" t="inlineStr"/>
-      <c r="E436" s="5" t="inlineStr"/>
+      <c r="E436" s="5" t="inlineStr">
+        <is>
+          <t>25/26 Sh/A 159</t>
+        </is>
+      </c>
       <c r="F436" s="5" t="inlineStr"/>
       <c r="G436" s="5" t="inlineStr">
         <is>
@@ -40761,7 +41303,11 @@
         </is>
       </c>
       <c r="D437" s="10" t="inlineStr"/>
-      <c r="E437" s="11" t="inlineStr"/>
+      <c r="E437" s="11" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 177</t>
+        </is>
+      </c>
       <c r="F437" s="11" t="inlineStr"/>
       <c r="G437" s="11" t="inlineStr">
         <is>
@@ -40926,7 +41472,7 @@
       </c>
       <c r="T438" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 88 336-77-74 / +998 90 716-31-42 (Onasi)</t>
         </is>
       </c>
       <c r="U438" s="7" t="inlineStr">
@@ -41034,7 +41580,7 @@
       </c>
       <c r="T439" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 95 583-88-58 / +998 91 641-75-32 (Onasi)</t>
         </is>
       </c>
       <c r="U439" s="17" t="inlineStr">
@@ -41321,7 +41867,11 @@
         </is>
       </c>
       <c r="D443" s="10" t="inlineStr"/>
-      <c r="E443" s="11" t="inlineStr"/>
+      <c r="E443" s="11" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A94</t>
+        </is>
+      </c>
       <c r="F443" s="11" t="inlineStr"/>
       <c r="G443" s="11" t="inlineStr">
         <is>
@@ -41566,7 +42116,7 @@
       </c>
       <c r="T445" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 586-06-97 / +998 88 585-14-06 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U445" s="7" t="inlineStr">
@@ -41601,7 +42151,11 @@
         </is>
       </c>
       <c r="D446" s="4" t="inlineStr"/>
-      <c r="E446" s="5" t="inlineStr"/>
+      <c r="E446" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A 98</t>
+        </is>
+      </c>
       <c r="F446" s="5" t="inlineStr"/>
       <c r="G446" s="5" t="inlineStr">
         <is>
@@ -41739,7 +42293,7 @@
       </c>
       <c r="E448" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>26/27 sh/a 100</t>
         </is>
       </c>
       <c r="F448" s="5" t="inlineStr">
@@ -41806,7 +42360,7 @@
       </c>
       <c r="T448" s="5" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>+998 91 464-92-28 / +998 88 601-52-00 (Onasi)</t>
         </is>
       </c>
       <c r="U448" s="7" t="inlineStr">
@@ -42005,7 +42559,11 @@
         </is>
       </c>
       <c r="D451" s="10" t="inlineStr"/>
-      <c r="E451" s="11" t="inlineStr"/>
+      <c r="E451" s="11" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A 103</t>
+        </is>
+      </c>
       <c r="F451" s="11" t="inlineStr"/>
       <c r="G451" s="11" t="inlineStr">
         <is>
@@ -42166,7 +42724,7 @@
       </c>
       <c r="T452" s="5" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>+998 94 333-76-08 / +998 94 330-22-74 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U452" s="7" t="inlineStr">
@@ -42207,7 +42765,7 @@
       </c>
       <c r="E453" s="11" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>26/27 SH/A105</t>
         </is>
       </c>
       <c r="F453" s="11" t="inlineStr">
@@ -42282,7 +42840,7 @@
       </c>
       <c r="T453" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 485-36-08 / +998 97 188-07-57 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U453" s="7" t="inlineStr">
@@ -42317,7 +42875,11 @@
         </is>
       </c>
       <c r="D454" s="4" t="inlineStr"/>
-      <c r="E454" s="5" t="inlineStr"/>
+      <c r="E454" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A106</t>
+        </is>
+      </c>
       <c r="F454" s="5" t="inlineStr"/>
       <c r="G454" s="5" t="inlineStr">
         <is>
@@ -42407,7 +42969,7 @@
       </c>
       <c r="E455" s="11" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>25/26 SH/A 229</t>
         </is>
       </c>
       <c r="F455" s="11" t="inlineStr">
@@ -42472,11 +43034,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T455" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T455" s="11" t="inlineStr"/>
       <c r="U455" s="15" t="inlineStr">
         <is>
           <t>CHALA</t>
@@ -42902,7 +43460,7 @@
       </c>
       <c r="T460" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 633-04-14 / +998 91 470-59-57 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U460" s="7" t="inlineStr">
@@ -43016,11 +43574,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T461" s="11" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="T461" s="11" t="inlineStr"/>
       <c r="U461" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -43053,7 +43607,11 @@
         </is>
       </c>
       <c r="D462" s="4" t="inlineStr"/>
-      <c r="E462" s="5" t="inlineStr"/>
+      <c r="E462" s="5" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A114</t>
+        </is>
+      </c>
       <c r="F462" s="5" t="inlineStr"/>
       <c r="G462" s="5" t="inlineStr">
         <is>
@@ -43464,11 +44022,7 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="T466" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T466" s="5" t="inlineStr"/>
       <c r="U466" s="15" t="inlineStr">
         <is>
           <t>CHALA</t>
@@ -43846,7 +44400,7 @@
       </c>
       <c r="T470" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 59 390-70-50 / +998 99 143-79-03 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U470" s="7" t="inlineStr">
@@ -43887,7 +44441,7 @@
       </c>
       <c r="E471" s="11" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>26/27 SH/A123</t>
         </is>
       </c>
       <c r="F471" s="11" t="inlineStr">
@@ -43962,7 +44516,7 @@
       </c>
       <c r="T471" s="11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 91 960-08-14 / +998 91 225-07-67 (Onasi)</t>
         </is>
       </c>
       <c r="U471" s="7" t="inlineStr">
@@ -43999,7 +44553,7 @@
       <c r="D472" s="4" t="inlineStr"/>
       <c r="E472" s="5" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>26/27 SH/A174</t>
         </is>
       </c>
       <c r="F472" s="5" t="inlineStr">
@@ -44072,11 +44626,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T472" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T472" s="5" t="inlineStr"/>
       <c r="U472" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -44109,7 +44659,11 @@
         </is>
       </c>
       <c r="D473" s="10" t="inlineStr"/>
-      <c r="E473" s="11" t="inlineStr"/>
+      <c r="E473" s="11" t="inlineStr">
+        <is>
+          <t>26/37 SH/A 125</t>
+        </is>
+      </c>
       <c r="F473" s="11" t="inlineStr"/>
       <c r="G473" s="11" t="inlineStr">
         <is>
@@ -44250,7 +44804,7 @@
       </c>
       <c r="T474" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 77 809-82-30 / +998 99 565-86-81 (Onasi)</t>
         </is>
       </c>
       <c r="U474" s="7" t="inlineStr">
@@ -44444,7 +44998,7 @@
       </c>
       <c r="T476" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 97 573-22-92</t>
         </is>
       </c>
       <c r="U476" s="7" t="inlineStr">
@@ -44804,7 +45358,7 @@
       </c>
       <c r="T480" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 70 290-27-40 / +998 88 263-38-33 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U480" s="5" t="inlineStr"/>
@@ -44837,7 +45391,7 @@
       </c>
       <c r="E481" s="11" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>25/26 SH/A 264</t>
         </is>
       </c>
       <c r="F481" s="11" t="inlineStr">
@@ -44910,11 +45464,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T481" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="T481" s="11" t="inlineStr"/>
       <c r="U481" s="7" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -45121,7 +45671,7 @@
       <c r="D484" s="4" t="inlineStr"/>
       <c r="E484" s="5" t="inlineStr">
         <is>
-          <t>298</t>
+          <t>25/26 Sh/A 266</t>
         </is>
       </c>
       <c r="F484" s="12" t="n">
@@ -45186,7 +45736,7 @@
       </c>
       <c r="T484" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>+998 87 561-52-96 / +998 77 232-28-78 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U484" s="15" t="inlineStr">
@@ -45225,7 +45775,11 @@
         </is>
       </c>
       <c r="D485" s="10" t="inlineStr"/>
-      <c r="E485" s="11" t="inlineStr"/>
+      <c r="E485" s="11" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 272</t>
+        </is>
+      </c>
       <c r="F485" s="11" t="inlineStr"/>
       <c r="G485" s="11" t="inlineStr">
         <is>
@@ -45399,7 +45953,7 @@
       </c>
       <c r="E487" s="11" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>25/26 SH/A 369</t>
         </is>
       </c>
       <c r="F487" s="11" t="inlineStr">
@@ -45474,7 +46028,7 @@
       </c>
       <c r="T487" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 50 501-01-82 / +998 88 078-06-86 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U487" s="7" t="inlineStr">
@@ -45670,7 +46224,7 @@
       </c>
       <c r="T489" s="11" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>+998 70 072-06-14 / +998 95 774-15-64 (Onasi)</t>
         </is>
       </c>
       <c r="U489" s="15" t="inlineStr">
@@ -46028,7 +46582,7 @@
       </c>
       <c r="T493" s="11" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>+998 97 066-26-92</t>
         </is>
       </c>
       <c r="U493" s="7" t="inlineStr">
@@ -46067,7 +46621,11 @@
         </is>
       </c>
       <c r="D494" s="4" t="inlineStr"/>
-      <c r="E494" s="5" t="inlineStr"/>
+      <c r="E494" s="5" t="inlineStr">
+        <is>
+          <t>26/27 sh/a 147</t>
+        </is>
+      </c>
       <c r="F494" s="5" t="inlineStr"/>
       <c r="G494" s="5" t="inlineStr">
         <is>
@@ -46151,7 +46709,11 @@
         </is>
       </c>
       <c r="D495" s="10" t="inlineStr"/>
-      <c r="E495" s="11" t="inlineStr"/>
+      <c r="E495" s="11" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 263</t>
+        </is>
+      </c>
       <c r="F495" s="11" t="inlineStr"/>
       <c r="G495" s="11" t="inlineStr">
         <is>
@@ -46316,7 +46878,7 @@
       </c>
       <c r="T496" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 87 000-46-08 / +998 77 108-80-48 (Onasi)</t>
         </is>
       </c>
       <c r="U496" s="7" t="inlineStr">
@@ -46437,7 +46999,7 @@
       <c r="D498" s="4" t="inlineStr"/>
       <c r="E498" s="5" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>25/26 Sh/A 260</t>
         </is>
       </c>
       <c r="F498" s="5" t="inlineStr">
@@ -46512,7 +47074,7 @@
       </c>
       <c r="T498" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 87 631-07-21 / +998 87 528-07-82 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U498" s="7" t="inlineStr">
@@ -46635,7 +47197,11 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E500" s="5" t="inlineStr"/>
+      <c r="E500" s="5" t="inlineStr">
+        <is>
+          <t>26/27 SH/A153</t>
+        </is>
+      </c>
       <c r="F500" s="5" t="inlineStr"/>
       <c r="G500" s="5" t="inlineStr">
         <is>
@@ -46811,7 +47377,11 @@
         </is>
       </c>
       <c r="D502" s="4" t="inlineStr"/>
-      <c r="E502" s="5" t="inlineStr"/>
+      <c r="E502" s="5" t="inlineStr">
+        <is>
+          <t>26/27 sh/a 155</t>
+        </is>
+      </c>
       <c r="F502" s="5" t="inlineStr"/>
       <c r="G502" s="5" t="inlineStr">
         <is>
@@ -46970,7 +47540,7 @@
       </c>
       <c r="T503" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 85 872-70-10 / +998 06 872-08-85 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U503" s="7" t="inlineStr">
@@ -47153,7 +47723,7 @@
       <c r="S505" s="11" t="inlineStr"/>
       <c r="T505" s="11" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>+998 71 160-30-30</t>
         </is>
       </c>
       <c r="U505" s="15" t="inlineStr">
@@ -47362,7 +47932,7 @@
       </c>
       <c r="E508" s="5" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>26/27 SH/A 161</t>
         </is>
       </c>
       <c r="F508" s="5" t="inlineStr">
@@ -47437,7 +48007,7 @@
       </c>
       <c r="T508" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 89 818-38-00 / +998 88 386-17-12 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U508" s="7" t="inlineStr">
@@ -47712,7 +48282,11 @@
         </is>
       </c>
       <c r="D512" s="4" t="inlineStr"/>
-      <c r="E512" s="5" t="inlineStr"/>
+      <c r="E512" s="5" t="inlineStr">
+        <is>
+          <t>26/27 Sh/A165</t>
+        </is>
+      </c>
       <c r="F512" s="5" t="inlineStr"/>
       <c r="G512" s="5" t="inlineStr">
         <is>
@@ -47886,7 +48460,7 @@
       </c>
       <c r="E514" s="5" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>25/26 Sh/A246</t>
         </is>
       </c>
       <c r="F514" s="5" t="inlineStr">
@@ -47957,7 +48531,7 @@
       </c>
       <c r="T514" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 619-91-21</t>
         </is>
       </c>
       <c r="U514" s="7" t="inlineStr">
@@ -48151,8 +48725,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T516" s="5" t="n">
-        <v>2019</v>
+      <c r="T516" s="5" t="inlineStr">
+        <is>
+          <t>+998 88 385-13-78 / +998 88 418-82-78 (Otasi / Onasi)</t>
+        </is>
       </c>
       <c r="U516" s="7" t="inlineStr">
         <is>
@@ -48274,7 +48850,11 @@
         </is>
       </c>
       <c r="D518" s="4" t="inlineStr"/>
-      <c r="E518" s="5" t="inlineStr"/>
+      <c r="E518" s="5" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 338</t>
+        </is>
+      </c>
       <c r="F518" s="5" t="inlineStr"/>
       <c r="G518" s="5" t="inlineStr">
         <is>
@@ -48687,7 +49267,7 @@
       </c>
       <c r="T522" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 86 233-80-80 / +998 77 021-67-05 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U522" s="7" t="inlineStr">
@@ -48807,7 +49387,7 @@
       </c>
       <c r="T523" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 95 147-08-25 / +998 99 742-24-73 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U523" s="7" t="inlineStr">
@@ -48919,7 +49499,7 @@
       </c>
       <c r="T524" s="5" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>+998 99 559-09-30 / +998 95 182-01-95 (O'zi)</t>
         </is>
       </c>
       <c r="U524" s="7" t="inlineStr">
@@ -48964,7 +49544,7 @@
       </c>
       <c r="E525" s="11" t="inlineStr">
         <is>
-          <t>307</t>
+          <t>26/27 SH/A178</t>
         </is>
       </c>
       <c r="F525" s="11" t="inlineStr">
@@ -49037,8 +49617,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T525" s="11" t="n">
-        <v>2026</v>
+      <c r="T525" s="11" t="inlineStr">
+        <is>
+          <t>+998 87 934-03-01 / +998 88 722-88-84 (Onasi)</t>
+        </is>
       </c>
       <c r="U525" s="7" t="inlineStr">
         <is>
@@ -49153,7 +49735,7 @@
       </c>
       <c r="T526" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 90 881-06-10 / +998 90 863-16-74 (Onasi)</t>
         </is>
       </c>
       <c r="U526" s="7" t="inlineStr">
@@ -49188,7 +49770,11 @@
         </is>
       </c>
       <c r="D527" s="10" t="inlineStr"/>
-      <c r="E527" s="11" t="inlineStr"/>
+      <c r="E527" s="11" t="inlineStr">
+        <is>
+          <t>26/27 sh/a 180</t>
+        </is>
+      </c>
       <c r="F527" s="11" t="inlineStr"/>
       <c r="G527" s="11" t="inlineStr">
         <is>
@@ -49610,7 +50196,7 @@
       </c>
       <c r="E532" s="5" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>25/26 Sh/A367</t>
         </is>
       </c>
       <c r="F532" s="5" t="inlineStr"/>
@@ -49673,7 +50259,7 @@
       </c>
       <c r="T532" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 88 833-85-93 / +998 88 804-06-91 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U532" s="5" t="inlineStr"/>
@@ -49700,7 +50286,11 @@
         </is>
       </c>
       <c r="D533" s="10" t="inlineStr"/>
-      <c r="E533" s="11" t="inlineStr"/>
+      <c r="E533" s="11" t="inlineStr">
+        <is>
+          <t>25/26 SH/A 375</t>
+        </is>
+      </c>
       <c r="F533" s="11" t="inlineStr"/>
       <c r="G533" s="11" t="inlineStr">
         <is>
@@ -49865,7 +50455,7 @@
       </c>
       <c r="T534" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 041-02-27 / +998 88 170-80-81 (Otasi)</t>
         </is>
       </c>
       <c r="U534" s="7" t="inlineStr">
@@ -49965,7 +50555,7 @@
       </c>
       <c r="T535" s="11" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>+998 97 960-25-35 / +998 91 216-23-04 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U535" s="11" t="inlineStr"/>
@@ -50067,7 +50657,7 @@
       </c>
       <c r="T536" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>+998 33 380-11-21 / +998 88 009-61-66 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U536" s="7" t="inlineStr">
@@ -50183,7 +50773,7 @@
       </c>
       <c r="T537" s="11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>+998 06 816-17-70 / +998 96 166-08-83 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U537" s="7" t="inlineStr">
@@ -50224,7 +50814,7 @@
       </c>
       <c r="E538" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25/26 sh/a 333</t>
         </is>
       </c>
       <c r="F538" s="5" t="inlineStr">
@@ -50295,7 +50885,7 @@
       </c>
       <c r="T538" s="5" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>+998 70 088-02-80 / +998 88 028-08-80 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U538" s="7" t="inlineStr">
@@ -50334,7 +50924,11 @@
         </is>
       </c>
       <c r="D539" s="10" t="inlineStr"/>
-      <c r="E539" s="11" t="inlineStr"/>
+      <c r="E539" s="11" t="inlineStr">
+        <is>
+          <t>25/26 sh/a 33</t>
+        </is>
+      </c>
       <c r="F539" s="11" t="inlineStr"/>
       <c r="G539" s="11" t="inlineStr">
         <is>
@@ -50495,7 +51089,7 @@
       </c>
       <c r="T540" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 88 729-14-01 / +998 97 619-84-84 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U540" s="7" t="inlineStr">
@@ -50695,7 +51289,7 @@
       </c>
       <c r="T542" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 77 371-00-28 / +998 95 665-28-82 (Onasi)</t>
         </is>
       </c>
       <c r="U542" s="7" t="inlineStr">
@@ -50814,7 +51408,11 @@
         </is>
       </c>
       <c r="D544" s="4" t="inlineStr"/>
-      <c r="E544" s="5" t="inlineStr"/>
+      <c r="E544" s="5" t="inlineStr">
+        <is>
+          <t>25/26 SH/A358</t>
+        </is>
+      </c>
       <c r="F544" s="5" t="inlineStr"/>
       <c r="G544" s="5" t="inlineStr">
         <is>
@@ -50975,7 +51573,7 @@
       </c>
       <c r="T545" s="11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 88 079-07-24</t>
         </is>
       </c>
       <c r="U545" s="7" t="inlineStr">
@@ -51180,7 +51778,7 @@
       </c>
       <c r="E548" s="5" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>25/26 Sh/A361</t>
         </is>
       </c>
       <c r="F548" s="5" t="inlineStr">
@@ -51251,7 +51849,7 @@
       </c>
       <c r="T548" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 04 891-30-00 / +998 90 870-88-27 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U548" s="7" t="inlineStr">
@@ -51454,7 +52052,11 @@
         </is>
       </c>
       <c r="D551" s="10" t="inlineStr"/>
-      <c r="E551" s="11" t="inlineStr"/>
+      <c r="E551" s="11" t="inlineStr">
+        <is>
+          <t>25/26 Sh/A 346</t>
+        </is>
+      </c>
       <c r="F551" s="11" t="inlineStr"/>
       <c r="G551" s="11" t="inlineStr">
         <is>
@@ -51538,7 +52140,11 @@
         </is>
       </c>
       <c r="D552" s="4" t="inlineStr"/>
-      <c r="E552" s="5" t="inlineStr"/>
+      <c r="E552" s="5" t="inlineStr">
+        <is>
+          <t>25/26 Sh/A365</t>
+        </is>
+      </c>
       <c r="F552" s="5" t="inlineStr"/>
       <c r="G552" s="5" t="inlineStr">
         <is>
@@ -51876,7 +52482,7 @@
       </c>
       <c r="E556" s="5" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>25/26 SH/A 372</t>
         </is>
       </c>
       <c r="F556" s="5" t="inlineStr">
@@ -51951,7 +52557,7 @@
       </c>
       <c r="T556" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 75 613-00-20 / +998 05 181-88-40 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U556" s="7" t="inlineStr">
@@ -52051,7 +52657,7 @@
       </c>
       <c r="T557" s="11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 99 540-78-43 / +998 91 775-05-59 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U557" s="7" t="inlineStr">
@@ -52251,7 +52857,7 @@
       </c>
       <c r="T559" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>+998 33 115-80-83 / +998 97 618-83-80 (Otasi / Onasi)</t>
         </is>
       </c>
       <c r="U559" s="7" t="inlineStr">
@@ -52452,7 +53058,7 @@
       <c r="D562" s="4" t="inlineStr"/>
       <c r="E562" s="5" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>25/26 SH/A 511</t>
         </is>
       </c>
       <c r="F562" s="5" t="inlineStr">
@@ -52527,7 +53133,7 @@
       </c>
       <c r="T562" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>+998 88 123-65-47</t>
         </is>
       </c>
       <c r="U562" s="7" t="inlineStr">
@@ -52562,7 +53168,11 @@
         </is>
       </c>
       <c r="D563" s="10" t="inlineStr"/>
-      <c r="E563" s="11" t="inlineStr"/>
+      <c r="E563" s="11" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
       <c r="F563" s="11" t="inlineStr"/>
       <c r="G563" s="11" t="inlineStr">
         <is>

</xml_diff>